<commit_message>
fix: expose family/series/thickness_mm in aluminum profile Excel import
Review finding 4 (Important): parseAluminumProfileSheet already read the
new family/series/thickness_mm columns, but nothing else in the import
path exposed them:

- public/templates/TEMPLATE_หน้าตัดอลูมิเนียม.xlsx (regenerated via
  scripts/generate-inventory-templates.cjs) still only had the original
  3 columns, so there was no way to fill in the new fields via the
  downloadable template.
- The import preview table in ExcelUpload.jsx only rendered the
  original 3 columns/colSpan, silently hiding the new fields from the
  pre-import review step.

Extends the template headers/hints and the preview thead/tbody/colSpan
to 6 columns so the feature is usable end to end.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AMQaXDxhpxPz9aaj4gMSVD
</commit_message>
<xml_diff>
--- a/public/templates/TEMPLATE_หน้าตัดอลูมิเนียม.xlsx
+++ b/public/templates/TEMPLATE_หน้าตัดอลูมิเนียม.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:F4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -414,6 +414,15 @@
       <c r="C3" t="str">
         <v>ความยาวมาตรฐาน (เมตร)</v>
       </c>
+      <c r="D3" t="str">
+        <v>กลุ่มหน้าตัด</v>
+      </c>
+      <c r="E3" t="str">
+        <v>รุ่น/ซีรีส์</v>
+      </c>
+      <c r="F3" t="str">
+        <v>ความหนา (มม.)</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -425,10 +434,19 @@
       <c r="C4" t="str">
         <v>เช่น 6.4 (เว้นว่างได้ ค่าเริ่มต้น 6.4)</v>
       </c>
+      <c r="D4" t="str">
+        <v>เช่น กล่องร่อง (สำหรับผูกกับ BOM Template)</v>
+      </c>
+      <c r="E4" t="str">
+        <v>เช่น ทั่วไป, ยูโร, วิสดอม</v>
+      </c>
+      <c r="F4" t="str">
+        <v>เช่น 1.2</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>